<commit_message>
feat: use master district and taluka for entry
</commit_message>
<xml_diff>
--- a/samples/is_regular_master_sample.xlsx
+++ b/samples/is_regular_master_sample.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R122e7f651e4040b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" r:id="Re5e5f6d37de14d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc1d0c773581a4a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="2" r:id="R1c816c432ef443c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -446,6 +446,8 @@
     <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="20" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -543,6 +545,12 @@
       </x:c>
       <x:c r="U1" s="5" t="str">
         <x:v>VILLAGE</x:v>
+      </x:c>
+      <x:c r="V1" s="5" t="str">
+        <x:v>DISTRICT</x:v>
+      </x:c>
+      <x:c r="W1" s="5" t="str">
+        <x:v>TALUKA</x:v>
       </x:c>
     </x:row>
     <x:row r="2">

</xml_diff>